<commit_message>
feat: update revenue calculation and formatting in summary report
</commit_message>
<xml_diff>
--- a/contoh/20260414 - KSC - AYO v4.xlsx
+++ b/contoh/20260414 - KSC - AYO v4.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="22">
   <si>
     <t xml:space="preserve">REVENUE KSC DAILY: &lt;&lt;&gt;&gt;</t>
   </si>
@@ -63,10 +63,19 @@
 Rp</t>
   </si>
   <si>
-    <t xml:space="preserve">1. MONTHLY MEMBERSHIP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. ACADEMY TENNIS</t>
+    <t xml:space="preserve">1. LES RENANG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. RENANG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. GYM CLASS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. GYM CLASS, RENANG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. ACADEMY TENNIS</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL MONTHLY MEMBERSHIP REVENUE (&lt;&lt;&gt;&gt;)</t>
@@ -273,7 +282,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="31">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -358,8 +367,16 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -640,7 +657,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B2:D18"/>
+  <dimension ref="B2:D21"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="45.68"/>
@@ -735,53 +752,77 @@
       <c r="D12" s="20"/>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="21" t="s">
         <v>13</v>
       </c>
       <c r="C13" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="D13" s="21"/>
+      <c r="D13" s="22"/>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="C14" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="D14" s="21"/>
+      <c r="C14" s="7" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="22" t="s">
+      <c r="B15" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="C15" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="D15" s="13" t="s">
+      <c r="C15" s="7" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="21" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="23"/>
-      <c r="C16" s="24"/>
-      <c r="D16" s="21"/>
+      <c r="C16" s="7" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="25" t="s">
+      <c r="B17" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="C17" s="26" t="s">
-        <v>3</v>
-      </c>
-      <c r="D17" s="13" t="s">
+      <c r="C17" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="D17" s="22"/>
+    </row>
+    <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="24" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="27"/>
-      <c r="C18" s="28" t="s">
+      <c r="C18" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="D18" s="13" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B19" s="25"/>
+      <c r="C19" s="26"/>
+      <c r="D19" s="22"/>
+    </row>
+    <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B20" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="C20" s="28" t="s">
+        <v>3</v>
+      </c>
+      <c r="D20" s="13" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B21" s="29"/>
+      <c r="C21" s="30" t="s">
         <v>3</v>
       </c>
     </row>

</xml_diff>